<commit_message>
Arua Accounting System v0.8 - Complete Sample Business Workflow
</commit_message>
<xml_diff>
--- a/tests/SampleBusinessData/AruaDemoTrading/AruaDemoTrading.xlsx
+++ b/tests/SampleBusinessData/AruaDemoTrading/AruaDemoTrading.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reb498dc8adb6421f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="2" r:id="Redd899644a5240bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Manifest" sheetId="3" r:id="R76f249b4343f492d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7a6ad3765ce742dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="2" r:id="R24e13147da144706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Manifest" sheetId="3" r:id="Ra7c11b7440be4087"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -387,58 +387,106 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>Sales invoices</x:v>
+        <x:v>Sales quotations</x:v>
       </x:c>
       <x:c r="B12" s="2" t="n">
-        <x:v>360</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>Sales invoice lines</x:v>
+        <x:v>Sales quotation lines</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:v>900</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>Customer receipts</x:v>
+        <x:v>Sales orders</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
-        <x:v>240</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:v>Supplier bills</x:v>
+        <x:v>Sales order lines</x:v>
       </x:c>
       <x:c r="B15" s="2" t="n">
-        <x:v>190</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>Supplier bill lines</x:v>
+        <x:v>Sales invoices</x:v>
       </x:c>
       <x:c r="B16" s="2" t="n">
-        <x:v>381</x:v>
+        <x:v>360</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>Supplier payments</x:v>
+        <x:v>Sales invoice lines</x:v>
       </x:c>
       <x:c r="B17" s="2" t="n">
-        <x:v>140</x:v>
+        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>Bank statement rows</x:v>
+        <x:v>Customer receipts</x:v>
       </x:c>
       <x:c r="B18" s="2" t="n">
-        <x:v>542</x:v>
+        <x:v>240</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>Purchase orders</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>Purchase order lines</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>Supplier bills</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="n">
+        <x:v>190</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>Supplier bill lines</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="n">
+        <x:v>381</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="2" t="str">
+        <x:v>Supplier credits (reference)</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="2" t="str">
+        <x:v>Supplier payments</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="n">
+        <x:v>140</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -671,27 +719,27 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>01_company_setup_reference.csv</x:v>
+        <x:v>00_accounting_entity_import.csv</x:v>
       </x:c>
       <x:c r="B2" s="2" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
-        <x:v>Reference/manual workflow</x:v>
+        <x:v>accounting entity import</x:v>
       </x:c>
       <x:c r="E2" s="2" t="str">
-        <x:v>Manual entity setup reference</x:v>
+        <x:v>Creates the sample Company through the standard entity workflow</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>02_branches_reference.csv</x:v>
+        <x:v>01_company_setup_reference.csv</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
         <x:v>No</x:v>
@@ -700,15 +748,15 @@
         <x:v>Reference/manual workflow</x:v>
       </x:c>
       <x:c r="E3" s="2" t="str">
-        <x:v>Manual branch setup reference</x:v>
+        <x:v>Manual entity setup reference</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>02_tax_setup_reference.csv</x:v>
+        <x:v>02_branches_reference.csv</x:v>
       </x:c>
       <x:c r="B4" s="2" t="n">
-        <x:v>12</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="2" t="str">
         <x:v>No</x:v>
@@ -717,151 +765,151 @@
         <x:v>Reference/manual workflow</x:v>
       </x:c>
       <x:c r="E4" s="2" t="str">
-        <x:v>Generic v0.7 tax setup reference; not an NZ return configuration</x:v>
+        <x:v>Manual branch setup reference</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>03_chart_of_accounts.csv</x:v>
+        <x:v>02_tax_setup_reference.csv</x:v>
       </x:c>
       <x:c r="B5" s="2" t="n">
-        <x:v>34</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="D5" s="2" t="str">
-        <x:v>chart_of_accounts</x:v>
+        <x:v>Reference/manual workflow</x:v>
       </x:c>
       <x:c r="E5" s="2" t="str">
-        <x:v>Adds 34 accounts to the six system accounts created with the entity</x:v>
+        <x:v>Generic v0.7 tax setup reference; not an NZ return configuration</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>04_customers.csv</x:v>
+        <x:v>03_chart_of_accounts.csv</x:v>
       </x:c>
       <x:c r="B6" s="2" t="n">
-        <x:v>50</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C6" s="2" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
-        <x:v>customers</x:v>
+        <x:v>chart_of_accounts</x:v>
       </x:c>
       <x:c r="E6" s="2" t="str">
-        <x:v>Fifty fictional customers</x:v>
+        <x:v>Adds 34 accounts to the six system accounts created with the entity</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>05_suppliers.csv</x:v>
+        <x:v>04_customers.csv</x:v>
       </x:c>
       <x:c r="B7" s="2" t="n">
-        <x:v>25</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C7" s="2" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D7" s="2" t="str">
-        <x:v>suppliers</x:v>
+        <x:v>customers</x:v>
       </x:c>
       <x:c r="E7" s="2" t="str">
-        <x:v>Twenty-five fictional suppliers</x:v>
+        <x:v>Fifty fictional customers</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>06_products_services.csv</x:v>
+        <x:v>05_suppliers.csv</x:v>
       </x:c>
       <x:c r="B8" s="2" t="n">
-        <x:v>40</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>products</x:v>
+        <x:v>suppliers</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
-        <x:v>Twenty-four products and sixteen services</x:v>
+        <x:v>Twenty-five fictional suppliers</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>07_sales_invoices.csv</x:v>
+        <x:v>06_products_services.csv</x:v>
       </x:c>
       <x:c r="B9" s="2" t="n">
-        <x:v>900</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>sales_invoices</x:v>
+        <x:v>products</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
-        <x:v>Three hundred sixty grouped sales invoices</x:v>
+        <x:v>Twenty-four products and sixteen services</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>07_sales_invoice_summary_reference.csv</x:v>
+        <x:v>07a_sales_quotations.csv</x:v>
       </x:c>
       <x:c r="B10" s="2" t="n">
-        <x:v>360</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
-        <x:v>Reference/manual workflow</x:v>
+        <x:v>sales_quotations</x:v>
       </x:c>
       <x:c r="E10" s="2" t="str">
-        <x:v>Reference totals for validating imported grouped invoices</x:v>
+        <x:v>Three grouped draft quotations demonstrating multiple lines, branches, and discounts</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="2" t="str">
-        <x:v>08_customer_receipts_reference.csv</x:v>
+        <x:v>07b_sales_orders.csv</x:v>
       </x:c>
       <x:c r="B11" s="2" t="n">
-        <x:v>240</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
-        <x:v>Reference/manual workflow</x:v>
+        <x:v>sales_orders</x:v>
       </x:c>
       <x:c r="E11" s="2" t="str">
-        <x:v>REFERENCE DATA – CURRENTLY NOT DIRECTLY IMPORTABLE; enter through Sales receipts workflow</x:v>
+        <x:v>Three grouped draft sales orders aligned with the demonstration quotation story</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="2" t="str">
-        <x:v>09_supplier_bills.csv</x:v>
+        <x:v>07_sales_invoices.csv</x:v>
       </x:c>
       <x:c r="B12" s="2" t="n">
-        <x:v>381</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D12" s="2" t="str">
-        <x:v>supplier_bills</x:v>
+        <x:v>sales_invoices</x:v>
       </x:c>
       <x:c r="E12" s="2" t="str">
-        <x:v>One hundred ninety grouped supplier bills</x:v>
+        <x:v>Three hundred sixty grouped sales invoices</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>09_supplier_bill_summary_reference.csv</x:v>
+        <x:v>07_sales_invoice_summary_reference.csv</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:v>190</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
         <x:v>No</x:v>
@@ -870,15 +918,15 @@
         <x:v>Reference/manual workflow</x:v>
       </x:c>
       <x:c r="E13" s="2" t="str">
-        <x:v>Reference totals for validating imported grouped bills</x:v>
+        <x:v>Reference totals for validating imported grouped invoices</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>10_supplier_payments_reference.csv</x:v>
+        <x:v>08_customer_receipts_reference.csv</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
-        <x:v>140</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="C14" s="2" t="str">
         <x:v>No</x:v>
@@ -887,57 +935,142 @@
         <x:v>Reference/manual workflow</x:v>
       </x:c>
       <x:c r="E14" s="2" t="str">
-        <x:v>REFERENCE DATA – CURRENTLY NOT DIRECTLY IMPORTABLE; enter through Purchases payments workflow</x:v>
+        <x:v>REFERENCE DATA – CURRENTLY NOT DIRECTLY IMPORTABLE; enter through Sales receipts workflow</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:v>11_manual_journals.csv</x:v>
+        <x:v>09_supplier_bills.csv</x:v>
       </x:c>
       <x:c r="B15" s="2" t="n">
-        <x:v>80</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D15" s="2" t="str">
-        <x:v>manual_journals</x:v>
+        <x:v>supplier_bills</x:v>
       </x:c>
       <x:c r="E15" s="2" t="str">
-        <x:v>Forty balanced adjusting journals</x:v>
+        <x:v>One hundred ninety grouped supplier bills</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>12_bank_statement.csv</x:v>
+        <x:v>09_supplier_bill_summary_reference.csv</x:v>
       </x:c>
       <x:c r="B16" s="2" t="n">
-        <x:v>542</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="D16" s="2" t="str">
-        <x:v>existing v0.5 bank statement importer</x:v>
+        <x:v>Reference/manual workflow</x:v>
       </x:c>
       <x:c r="E16" s="2" t="str">
-        <x:v>Evidence-only statement; import creates no journals</x:v>
+        <x:v>Reference totals for validating imported grouped bills</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="2" t="str">
+        <x:v>09a_purchase_orders.csv</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>purchase_orders</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str">
+        <x:v>Three grouped draft purchase orders demonstrating multiple lines, branches, and discounts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>10a_supplier_credits_reference.csv</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Reference/manual workflow</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>REFERENCE DATA – enter through Purchases after the linked supplier bills are posted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>10_supplier_payments_reference.csv</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>Reference/manual workflow</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str">
+        <x:v>REFERENCE DATA – CURRENTLY NOT DIRECTLY IMPORTABLE; enter through Purchases payments workflow</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>11_manual_journals.csv</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>manual_journals</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>Forty balanced adjusting journals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>12_bank_statement.csv</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="n">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>existing v0.5 bank statement importer</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>Evidence-only statement; import creates no journals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="2" t="str">
         <x:v>13_opening_balances.csv</x:v>
       </x:c>
-      <x:c r="B17" s="2" t="n">
+      <x:c r="B22" s="2" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C17" s="2" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="D17" s="2" t="str">
+      <x:c r="C22" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
         <x:v>opening_balances</x:v>
       </x:c>
-      <x:c r="E17" s="2" t="str">
+      <x:c r="E22" s="2" t="str">
         <x:v>Balanced staging only; v0.8 cannot post this batch</x:v>
       </x:c>
     </x:row>

</xml_diff>